<commit_message>
Ajustado las matematicas del ejercicio
</commit_message>
<xml_diff>
--- a/Algoritmo Pillo Fon.xlsx
+++ b/Algoritmo Pillo Fon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ankes\Documents\Tareas\Programacion Basica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{238EBB3F-5944-4708-AE15-E7996C7A2FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E5FE04-CC55-483F-8A64-468CCC40C176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D7A16764-DA4C-4422-9899-B0AA0BF62451}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="86">
   <si>
     <t>Entrada</t>
   </si>
@@ -145,9 +145,6 @@
     <t>sueldoDiarioLV</t>
   </si>
   <si>
-    <t>HorasEmpleadoPlantaLV*SueldoEmpleadoHora</t>
-  </si>
-  <si>
     <t>"Sueldo Diario de Lunes a viernes"</t>
   </si>
   <si>
@@ -199,9 +196,6 @@
     <t>horasEmpleadoPlantaMesLV + horasEmpleadoPlantaSabadoMes</t>
   </si>
   <si>
-    <t>horasEmpleadoPlantaMes /2 * sueldoEmpleadoHora</t>
-  </si>
-  <si>
     <t>"Sueldo quincenal del Empleado de planta"</t>
   </si>
   <si>
@@ -214,20 +208,116 @@
     <t>horasEmpleadoMedioTiempoSemanalLS</t>
   </si>
   <si>
-    <t>horasEmpleadoMedioTiempoDiariaLS * 6 (39)</t>
-  </si>
-  <si>
-    <t>horasEmpleadoMedioTiempoSemanalLS*4 (156)</t>
-  </si>
-  <si>
     <t>horasEmpleadoMedioTiempoMes</t>
+  </si>
+  <si>
+    <t>Case 2: Empleado Medio Tiempo</t>
+  </si>
+  <si>
+    <t>horasEmpleadoMedioTiempoDiariaLS * 6 (33)</t>
+  </si>
+  <si>
+    <t>horasEmpleadoMedioTiempoSemanalLS*4 (132)</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoHora</t>
+  </si>
+  <si>
+    <t>sueldoMensual/horasEmpleadoMedioTiempoMes</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoS</t>
+  </si>
+  <si>
+    <t>horasEmpleadoMedioTiempoDiariaLS * sueldoEmpleadoMedioTiempoHora</t>
+  </si>
+  <si>
+    <t>horasEmpleadoPlantaLV*sueldoEmpleadoHora</t>
+  </si>
+  <si>
+    <t>horasEmpleadoMedioTiempoSemanalLS - 5.5 * sueldoEmpleadoMedioTiempoHora</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoHora / 60</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoMinuto</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoSegundo</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoSemanaLV</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoSemanaLS</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoQuincenal</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoMinuto / 60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horasEmpleadoMedioTiempoSemanaLS - 5.5 * sueldoEmpleadoMedioTiempoHora </t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoMedioTiempoHora * horasEmpleadoMedioTiempoSemanalLS</t>
+  </si>
+  <si>
+    <t>horasEmpleadoMedioTiempoMes /2 * sueldoEmpleadoMedioTiempoHora</t>
+  </si>
+  <si>
+    <t>horasEmpleadoPlantaMes /2 * sueldoEmpleadoPlantaHora</t>
+  </si>
+  <si>
+    <t>Case 3: Empleado Medio Tiempo</t>
+  </si>
+  <si>
+    <t>horasEmpleadoContratoSemanal</t>
+  </si>
+  <si>
+    <t>horasEmpleadoContratoSemanal &lt; 30 || horasEmpleadoContratoSemanal &gt; 40</t>
+  </si>
+  <si>
+    <t>“ERROR: horas fuera de rango permitido”</t>
+  </si>
+  <si>
+    <t>horasEmpleadoContratoMes</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoContratoHora</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoContratoMinuto</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoContratoSegundo</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoContratoQuincenal</t>
+  </si>
+  <si>
+    <t>sueldoMensual/horasEmpleadoContratoMes</t>
+  </si>
+  <si>
+    <t>horasEmpleadoContratoSemanal * 4</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoContratoHora/60</t>
+  </si>
+  <si>
+    <t>sueldoEmpleadoContratoMinuto/60</t>
+  </si>
+  <si>
+    <t>horasEmpleadoContratoMes / 2 * sueldoEmpleadoContratoHora</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -250,13 +340,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -271,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -283,6 +387,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,7 +704,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2268464B-F785-49BD-B9C3-9BAFFB02D439}">
-  <dimension ref="C4:E34"/>
+  <dimension ref="C4:E42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="35.88671875" customWidth="1"/>
@@ -670,7 +777,7 @@
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D10" s="1">
         <v>9.5</v>
@@ -694,10 +801,10 @@
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.3">
@@ -713,7 +820,7 @@
         <v>15</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="3:5" x14ac:dyDescent="0.3">
@@ -743,156 +850,225 @@
         <v>29</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="19" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="20" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="21" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" t="s">
         <v>38</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="22" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" t="s">
         <v>41</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="23" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C24" t="s">
-        <v>51</v>
-      </c>
-      <c r="D24" s="1">
-        <v>6.5</v>
-      </c>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="3:5" ht="18" x14ac:dyDescent="0.35">
+      <c r="C24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
     </row>
     <row r="25" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
+      </c>
+      <c r="D25" s="1">
+        <v>5.5</v>
       </c>
     </row>
     <row r="26" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C32" t="s">
-        <v>38</v>
-      </c>
-      <c r="D32" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="33" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C33" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="D33" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C34" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>48</v>
+        <v>65</v>
+      </c>
+      <c r="D34" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C35" t="s">
+        <v>66</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="3:5" ht="18" x14ac:dyDescent="0.35">
+      <c r="C36" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+    </row>
+    <row r="37" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C37" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" t="s">
+        <v>74</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C38" t="s">
+        <v>76</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C39" t="s">
+        <v>77</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="40" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C40" t="s">
+        <v>78</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C41" t="s">
+        <v>79</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C42" t="s">
+        <v>80</v>
+      </c>
+      <c r="D42" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C36:E36"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>